<commit_message>
Mise à jour URL portfolio dans tableau de synthèse
</commit_message>
<xml_diff>
--- a/assets/Tableau_synthese_NGUEMA_Oscar.xlsx
+++ b/assets/Tableau_synthese_NGUEMA_Oscar.xlsx
@@ -1398,7 +1398,7 @@
     <row r="5" ht="39.9" customHeight="1" thickBot="1">
       <c r="A5" s="61" t="inlineStr">
         <is>
-          <t>Adresse URL du portfolio : https://oscar-nguema.fr  (Portfolio BTS SIO SLAM)</t>
+          <t>Adresse URL du portfolio : https://koscar4.github.io  (Portfolio BTS SIO SLAM)</t>
         </is>
       </c>
       <c r="B5" s="62" t="n"/>
@@ -2236,12 +2236,12 @@
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:E3"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.1968503937007874" bottom="0.1968503937007874" header="0.5118110236220472" footer="0.5118110236220472"/>

</xml_diff>